<commit_message>
Registo de NC v02: atualiza NC-M3-14 e NC-M3-15 com os rascunhos v02 (PR #169 a #180)
NC-M3-14 passa a "Aberta - correção em curso" (Plano de Qualidade v02 em rascunho).
NC-M3-15 inclui a arquitetura, o modelo de dados e os documentos v01 ainda com F005/F007,
esclarece que as Issues GitHub #16, #18, #59 e #61 são I059, I061, I028 e I030
e assinala o prazo de executor de I059 (25/10/2026).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FJ4FqWF1hX4FXNtdipqpfU
</commit_message>
<xml_diff>
--- a/02-artefactos-de-qualidade-de-processo/02.06-nao-conformidades-e-acoes-corretivas/m3-registo-nao-conformidades-v02.xlsx
+++ b/02-artefactos-de-qualidade-de-processo/02.06-nao-conformidades-e-acoes-corretivas/m3-registo-nao-conformidades-v02.xlsx
@@ -1535,7 +1535,7 @@
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>Não alterar o v01. Preparar o Plano de Qualidade de Processo v02 com as tecnologias do Regulamento v02, os quality gates QG-01 a QG-08 e o âmbito v05. É uma nova versão de artefacto: informar o docente e acrescentar a linha à CCA (Regulamento UC v19, secção 7.3).</t>
+          <t>Não alterar o v01. Plano de Qualidade de Processo v02 preparado em rascunho (PR #174) com as tecnologias do Regulamento v02, os quality gates QG-01 a QG-08 e o âmbito v05; falta o grupo aprová-lo. É uma nova versão de artefacto: informar o docente e acrescentar a linha à CCA (Regulamento UC v19, secção 7.3; linha AD-011 no rascunho da CCA v08, PR #175).</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
@@ -1550,16 +1550,16 @@
       </c>
       <c r="L15" s="5" t="inlineStr">
         <is>
-          <t>Aberta</t>
+          <t>Aberta - correção em curso</t>
         </is>
       </c>
       <c r="M15" s="4" t="inlineStr">
         <is>
-          <t>Plano de Qualidade v01 (secções 4, 6.3 e 7) e Regulamento de grupo v02 (secção 11)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="114.5" customHeight="1">
+          <t>Plano de Qualidade v01 (secções 4, 6.3 e 7), Regulamento de grupo v02 (secção 11) e rascunho do Plano de Qualidade v02 (PR #174)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="223" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
           <t>NC-M3-15</t>
@@ -1577,12 +1577,12 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>m3-prototipo-baixa-fidelidade-v02.md (04.10); scripts SQL m3-v01 06-contas-e-pagamentos.sql e 07-internamento.sql (04.13); m3-plano-testes-backend-v01.md; Issues #16, #18, #59 e #61</t>
+          <t>m3-prototipo-baixa-fidelidade-v02.md (04.10); m3-plano-testes-backend-v01.md (03.01.01); documentação da API, casos de uso, modelos de classes e RTM v01 (04.03, 04.04, 04.07, 04.11); documentação da arquitetura v01 (04.05); modelo de dados v01 (04.06); scripts SQL m3-v01 06-contas-e-pagamentos.sql e 07-internamento.sql (04.13); Issues #16, #18, #59 e #61</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>Depois da Declaração de Âmbito v05 (F005 contas e pagamentos e F007 internamento fora do âmbito; 51 passam a 37 endpoints), continuam em documentos M3: 5 ecrãs no protótipo v02 (W14, W15, W17, W18 e M05); as tabelas e scripts de contas, pagamentos e internamento (6 das 22 tabelas); o plano de testes v01 (51 endpoints); e o texto de 4 Issues do Sprint 04 (I059, I061, I028 e I030).</t>
+          <t>Depois da Declaração de Âmbito v05 (F005 contas e pagamentos e F007 internamento fora do âmbito; 51 passam a 37 endpoints), continuam em documentos M2 e M3: 5 ecrãs no protótipo v02 (W14, W15, W17, W18 e M05); a API, os casos de uso (UC14, UC15 e UC18), os modelos de classes e a RTM v01; os módulos ARC-F005 e ARC-F007 e as tecnologias antigas (.NET 8, Flutter) na documentação da arquitetura v01; as tabelas e scripts de contas, pagamentos e internamento (6 das 22 tabelas); o plano de testes v01 (51 endpoints); e o texto de 4 Issues do Sprint 04 (GitHub #16, #18, #59 e #61, que são as Issues I059, I061, I028 e I030 do backlog).</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
@@ -1602,7 +1602,7 @@
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>Protótipo: ecrãs retirados nesta correção. Plano de testes: v02 em rascunho (PR #172). Backlog: v03 descontinua as 9 tarefas. Scripts SQL, modelo de dados e texto das Issues: decidir no Backlog Refinement de 27/10/2026 (nova versão ou nota de âmbito). Os PDF assinados não se alteram.</t>
+          <t>Protótipo: ecrãs retirados nesta correção. Rascunhos v02 em PR: modelo de classes backend (#169), API (#170), casos de uso (#171), plano de testes (#172), plano de qualidade (#174), modelos de classes web (#176) e mobile (#177), RTM (#178), especificação de requisitos (#179) e diagrama de sequência (#180). Backlog: v03 descontinua as 9 tarefas. Arquitetura, modelo de dados, scripts SQL (6 das 22 tabelas) e texto das Issues #16, #18, #59 e #61: decidir no Backlog Refinement de 27/10/2026 (nova versão ou nota de âmbito); a Issue #16 (I059) tem prazo de executor a 25/10/2026 e mapeia todas as tabelas dos scripts, por isso convém decidir antes. Os PDF assinados não se alteram.</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
@@ -1622,7 +1622,7 @@
       </c>
       <c r="M16" s="4" t="inlineStr">
         <is>
-          <t>Rascunhos v02 (PR #169 a #172), protótipo v02 corrigido (PR de correções) e backlog v03 (rascunho)</t>
+          <t>Rascunhos v02 (PR #169 a #180), protótipo v02 corrigido (PR #173) e backlog v03 (rascunho)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Registo de NC v02: NC-M3-15 cita o rascunho da arquitetura v02 (PR #181)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FJ4FqWF1hX4FXNtdipqpfU
</commit_message>
<xml_diff>
--- a/02-artefactos-de-qualidade-de-processo/02.06-nao-conformidades-e-acoes-corretivas/m3-registo-nao-conformidades-v02.xlsx
+++ b/02-artefactos-de-qualidade-de-processo/02.06-nao-conformidades-e-acoes-corretivas/m3-registo-nao-conformidades-v02.xlsx
@@ -1602,7 +1602,7 @@
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>Protótipo: ecrãs retirados nesta correção. Rascunhos v02 em PR: modelo de classes backend (#169), API (#170), casos de uso (#171), plano de testes (#172), plano de qualidade (#174), modelos de classes web (#176) e mobile (#177), RTM (#178), especificação de requisitos (#179) e diagrama de sequência (#180). Backlog: v03 descontinua as 9 tarefas. Arquitetura, modelo de dados, scripts SQL (6 das 22 tabelas) e texto das Issues #16, #18, #59 e #61: decidir no Backlog Refinement de 27/10/2026 (nova versão ou nota de âmbito); a Issue #16 (I059) tem prazo de executor a 25/10/2026 e mapeia todas as tabelas dos scripts, por isso convém decidir antes. Os PDF assinados não se alteram.</t>
+          <t>Protótipo: ecrãs retirados nesta correção. Rascunhos v02 em PR: modelo de classes backend (#169), API (#170), casos de uso (#171), plano de testes (#172), plano de qualidade (#174), modelos de classes web (#176) e mobile (#177), RTM (#178), especificação de requisitos (#179), diagrama de sequência (#180) e arquitetura (#181). Backlog: v03 descontinua as 9 tarefas. Modelo de dados, scripts SQL (6 das 22 tabelas) e texto das Issues #16, #18, #59 e #61: decidir no Backlog Refinement de 27/10/2026 (nova versão ou nota de âmbito); a Issue #16 (I059) tem prazo de executor a 25/10/2026 e mapeia todas as tabelas dos scripts, por isso convém decidir antes. Os PDF assinados não se alteram.</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
@@ -1622,7 +1622,7 @@
       </c>
       <c r="M16" s="4" t="inlineStr">
         <is>
-          <t>Rascunhos v02 (PR #169 a #180), protótipo v02 corrigido (PR #173) e backlog v03 (rascunho)</t>
+          <t>Rascunhos v02 (PR #169 a #181), protótipo v02 corrigido (PR #173) e backlog v03 (rascunho)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Registo de NC v02: NC-M3-09 e NC-M3-14 atualizadas à v02 do Regulamento assinada a 24/10
A 24/10/2026 o Regulamento do Grupo v02 passou a citar a ata de 23/10 (arquivada em 01.03) e a data de aprovação 24/10. A NC-M3-09 fica parcialmente corrigida e acrescenta a convocatória de 23/10 que não está na pasta; a NC-M3-14 indica a nova data.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FJ4FqWF1hX4FXNtdipqpfU
</commit_message>
<xml_diff>
--- a/02-artefactos-de-qualidade-de-processo/02.06-nao-conformidades-e-acoes-corretivas/m3-registo-nao-conformidades-v02.xlsx
+++ b/02-artefactos-de-qualidade-de-processo/02.06-nao-conformidades-e-acoes-corretivas/m3-registo-nao-conformidades-v02.xlsx
@@ -1157,7 +1157,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="161" customHeight="1">
+    <row r="10" ht="250" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>NC-M3-09</t>
@@ -1175,12 +1175,12 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>m3-regulamento-grupo-v02.pdf (e v01); 01.03-reunioes-de-grupo</t>
+          <t>m3-regulamento-grupo-v02.pdf (e v01); m3-20261023-reuniao-extraordinaria-ata-v01.pdf; 01.03-reunioes-de-grupo</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>O histórico de versões do Regulamento de grupo v02 (21/10/2026) indica como ata de aprovação "m3-s03-20261021-ata-alteracao-regulamento-v01.pdf". Esse ficheiro não existe em 01.03-reunioes-de-grupo e o nome não segue o padrão das reuniões extraordinárias (sem sprint, com "reuniao-extraordinaria-ata"). Nas v01 e v02, a ata de aprovação inicial é citada como "m1-20260925-controlo-final-milestone-ata-v01.pdf", mas o ficheiro arquivado chama-se "m1-s01-20260925-controlo-final-milestone-ata-v01.pdf".</t>
+          <t>A 24/10/2026 o histórico de versões do Regulamento de grupo v02 passou a indicar como ata de aprovação "m3-20261023-reuniao-extraordinaria-ata-v01.pdf", que existe em 01.03-reunioes-de-grupo e segue o padrão das reuniões extraordinárias: esta parte ficou resolvida. Continua por resolver: (a) nas v01 e v02 do Regulamento, a ata de aprovação inicial é citada como "m1-20260925-controlo-final-milestone-ata-v01.pdf", mas o ficheiro arquivado chama-se "m1-s01-20260925-controlo-final-milestone-ata-v01.pdf"; (b) a ata de 23/10/2026 cita como convocatória "m3-20261022-reuniao-extraordinaria-convocatoria-v01.pdf", que não está em 01.03-reunioes-de-grupo (só existe "m3-20261016-reuniao-extraordinaria-convocatoria-v01.pdf").</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
@@ -1195,12 +1195,12 @@
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>A ata que aprova o Regulamento de grupo v02 não está identificável no arquivo; a aprovação da alteração fica sem evidência localizável.</t>
+          <t>Quem abre o Regulamento ou a ata de 23/10 não encontra, com o nome indicado, a ata de aprovação inicial (v01) nem a convocatória da reunião de 23/10. A v02 já aponta para a ata correta.</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>Não alterar os PDF assinados. Localizar e arquivar a ata da reunião de alteração do regulamento com o nome do padrão (m3-&lt;data&gt;-reuniao-extraordinaria-ata-v01.pdf); se não existir, informar o docente. Registar na ata de 23/10/2026 a correspondência com os nomes citados.</t>
+          <t>Não alterar os PDF assinados. Arquivar em 01.03 a convocatória citada pela ata de 23/10 (m3-20261022-reuniao-extraordinaria-convocatoria-v01.pdf) ou, se o nome estiver errado, registar na próxima ata a correspondência com o ficheiro real. Registar também a correspondência do nome da ata m1 (m1-s01-20260925-controlo-final-milestone-ata-v01.pdf).</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
@@ -1215,12 +1215,12 @@
       </c>
       <c r="L10" s="5" t="inlineStr">
         <is>
-          <t>Aberta</t>
+          <t>Aberta - parcialmente corrigida (ata de 23/10/2026 arquivada)</t>
         </is>
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>Texto do PDF m3-regulamento-grupo-v02.pdf (secção 2.2, histórico de versões) e lista de ficheiros de 01.03-reunioes-de-grupo</t>
+          <t>Histórico de versões (secção 2.2) do m3-regulamento-grupo-v02.md em docs/S04 (24/10/2026), ata de 23/10/2026 e lista de ficheiros de 01.03-reunioes-de-grupo</t>
         </is>
       </c>
     </row>
@@ -1515,7 +1515,7 @@
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>O Plano de Qualidade de Processo (v01, M1) ficou desatualizado face ao Regulamento de grupo v02 (21/10/2026): indica .NET 8 e EF Core 8 no m3, React 18 com TypeScript 5.3 e Flutter 3.19 no m4, comandos de quality gate com Flutter, o SharePoint como ferramenta, os quality gates QG-01 a QG-07 (sem QG-08) e a verificação das funcionalidades F001 a F007 (F005 e F007 estão fora do âmbito desde a Declaração de Âmbito v05).</t>
+          <t>O Plano de Qualidade de Processo (v01, M1) ficou desatualizado face ao Regulamento de grupo v02 (assinado a 24/10/2026): indica .NET 8 e EF Core 8 no m3, React 18 com TypeScript 5.3 e Flutter 3.19 no m4, comandos de quality gate com Flutter, o SharePoint como ferramenta, os quality gates QG-01 a QG-07 (sem QG-08) e a verificação das funcionalidades F001 a F007 (F005 e F007 estão fora do âmbito desde a Declaração de Âmbito v05).</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
@@ -1525,7 +1525,7 @@
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>O Regulamento de grupo e o âmbito foram alterados em 20 e 21/10 sem atualizar o Plano de Qualidade.</t>
+          <t>O Regulamento de grupo e o âmbito foram alterados entre 20 e 24/10 sem atualizar o Plano de Qualidade.</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Registo de NC v02: NC-M3-15 regista o modelo de dados v02, os scripts m3-v02 executados e a decisão do Líder de 24/10
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FJ4FqWF1hX4FXNtdipqpfU
</commit_message>
<xml_diff>
--- a/02-artefactos-de-qualidade-de-processo/02.06-nao-conformidades-e-acoes-corretivas/m3-registo-nao-conformidades-v02.xlsx
+++ b/02-artefactos-de-qualidade-de-processo/02.06-nao-conformidades-e-acoes-corretivas/m3-registo-nao-conformidades-v02.xlsx
@@ -1602,7 +1602,7 @@
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>Protótipo: ecrãs retirados nesta correção. Rascunhos v02 em PR: modelo de classes backend (#169), API (#170), casos de uso (#171), plano de testes (#172), plano de qualidade (#174), modelos de classes web (#176) e mobile (#177), RTM (#178), especificação de requisitos (#179), diagrama de sequência (#180) e arquitetura (#181). Backlog: v03 descontinua as 9 tarefas. Modelo de dados, scripts SQL (6 das 22 tabelas) e texto das Issues #16, #18, #59 e #61: decidir no Backlog Refinement de 27/10/2026 (nova versão ou nota de âmbito); a Issue #16 (I059) tem prazo de executor a 25/10/2026 e mapeia todas as tabelas dos scripts, por isso convém decidir antes. Os PDF assinados não se alteram.</t>
+          <t>Protótipo: ecrãs retirados nesta correção. Rascunhos v02 em PR: modelo de classes backend (#169), API (#170), casos de uso (#171), plano de testes (#172), plano de qualidade (#174), modelos de classes web (#176) e mobile (#177), RTM (#178), especificação de requisitos (#179), diagrama de sequência (#180) e arquitetura (#181). Backlog: v03 descontinua as 9 tarefas. Modelo de dados v02 (#183) e scripts m3-v02 (#184): as 6 tabelas de F005 e F007 saem (ficam 16 tabelas), por decisão do Líder de 24/10/2026; os scripts m3-v02 foram executados num SQL Server 2025 a 24/10/2026 (237 verificações sem divergências e 41 testes de 41 com êxito). Texto das Issues #16, #18, #59 e #61: a Issue #16 (I059) tem prazo de executor a 25/10/2026 e o texto de decisão está pronto a colar na Issue; nas outras decide-se no Backlog Refinement de 27/10/2026 (nova versão ou nota de âmbito). Os PDF assinados não se alteram.</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
@@ -1622,7 +1622,7 @@
       </c>
       <c r="M16" s="4" t="inlineStr">
         <is>
-          <t>Rascunhos v02 (PR #169 a #181), protótipo v02 corrigido (PR #173) e backlog v03 (rascunho)</t>
+          <t>Rascunhos v02 (PR #169 a #181, #183 e #184), protótipo v02 corrigido (PR #173) e backlog v03 (rascunho)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Registo de NC v02: NC-M3-09 regista que a convocatória de 22/10 foi enviada e não tem PDF assinado (decisão do Líder de 25/10)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FJ4FqWF1hX4FXNtdipqpfU
</commit_message>
<xml_diff>
--- a/02-artefactos-de-qualidade-de-processo/02.06-nao-conformidades-e-acoes-corretivas/m3-registo-nao-conformidades-v02.xlsx
+++ b/02-artefactos-de-qualidade-de-processo/02.06-nao-conformidades-e-acoes-corretivas/m3-registo-nao-conformidades-v02.xlsx
@@ -1180,7 +1180,7 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>A 24/10/2026 o histórico de versões do Regulamento de grupo v02 passou a indicar como ata de aprovação "m3-20261023-reuniao-extraordinaria-ata-v01.pdf", que existe em 01.03-reunioes-de-grupo e segue o padrão das reuniões extraordinárias: esta parte ficou resolvida. Continua por resolver: (a) nas v01 e v02 do Regulamento, a ata de aprovação inicial é citada como "m1-20260925-controlo-final-milestone-ata-v01.pdf", mas o ficheiro arquivado chama-se "m1-s01-20260925-controlo-final-milestone-ata-v01.pdf"; (b) a ata de 23/10/2026 cita como convocatória "m3-20261022-reuniao-extraordinaria-convocatoria-v01.pdf", que não está em 01.03-reunioes-de-grupo (só existe "m3-20261016-reuniao-extraordinaria-convocatoria-v01.pdf").</t>
+          <t>A 24/10/2026 o histórico de versões do Regulamento de grupo v02 passou a indicar como ata de aprovação "m3-20261023-reuniao-extraordinaria-ata-v01.pdf", que existe em 01.03-reunioes-de-grupo e segue o padrão das reuniões extraordinárias: esta parte ficou resolvida. Continua por resolver: (a) nas v01 e v02 do Regulamento, a ata de aprovação inicial é citada como "m1-20260925-controlo-final-milestone-ata-v01.pdf", mas o ficheiro arquivado chama-se "m1-s01-20260925-controlo-final-milestone-ata-v01.pdf"; (b) a ata de 23/10/2026 cita como convocatória "m3-20261022-reuniao-extraordinaria-convocatoria-v01.pdf". A convocatória foi enviada a 22/10/2026 e não existe PDF assinado no repositório (em 01.03-reunioes-de-grupo só existe "m3-20261016-reuniao-extraordinaria-convocatoria-v01.pdf"). Por decisão do Líder de 25/10/2026, não vai ser assinada agora, porque já foi enviada e o prazo de envio passou.</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
@@ -1200,7 +1200,7 @@
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>Não alterar os PDF assinados. Arquivar em 01.03 a convocatória citada pela ata de 23/10 (m3-20261022-reuniao-extraordinaria-convocatoria-v01.pdf) ou, se o nome estiver errado, registar na próxima ata a correspondência com o ficheiro real. Registar também a correspondência do nome da ata m1 (m1-s01-20260925-controlo-final-milestone-ata-v01.pdf).</t>
+          <t>Não alterar os PDF assinados. Não assinar a convocatória de 22/10/2026 agora e registar na próxima ata o facto (enviada a 22/10/2026, sem PDF assinado no repositório). Registar também a correspondência do nome da ata m1 (m1-s01-20260925-controlo-final-milestone-ata-v01.pdf).</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">

</xml_diff>